<commit_message>
Overhaul soils data-entry form and sync field form
Vegetation work having shipped, this reworks the soils templates:

- Mottles split into three columns (mottle_abundance / mottle_size /
  mottle_contrast); standalone redox column removed (not on the field form).
- Added plot-level physiography to the Excel plots sheet: slope_position,
  slope_pct, aspect (8-point compass + Flat), drainage (CSSC 7-class
  VR/R/W/MW/I/P/VP), and surface_stones (S0-S5).
- horizon column restricted to a dropdown of CSSC horizon designations
  (union of cssc_great_groups.csv key_horizons + a wetland default set;
  letters only, no numbered subdivisions).
- Synced create_forms.py (soils PDF): CSSC 7-class drainage, compass
  aspect replacing the degrees field, physiography regrouped into 3 rows.
- Updated the soils ingest column-list comment to match.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/templates/soils_data_entry.xlsx
+++ b/inst/templates/soils_data_entry.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="88">
   <si>
     <t xml:space="preserve">SOILS FIELD DATA FORM  ·  Alberta Wetland Assessment</t>
   </si>
@@ -46,6 +46,21 @@
     <t xml:space="preserve">gps_northing</t>
   </si>
   <si>
+    <t xml:space="preserve">slope_position</t>
+  </si>
+  <si>
+    <t xml:space="preserve">slope_pct</t>
+  </si>
+  <si>
+    <t xml:space="preserve">aspect</t>
+  </si>
+  <si>
+    <t xml:space="preserve">drainage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">surface_stones</t>
+  </si>
+  <si>
     <t xml:space="preserve">hydric_ind_present</t>
   </si>
   <si>
@@ -85,6 +100,21 @@
     <t xml:space="preserve">5900000</t>
   </si>
   <si>
+    <t xml:space="preserve">L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S0</t>
+  </si>
+  <si>
     <t xml:space="preserve">Yes</t>
   </si>
   <si>
@@ -127,10 +157,13 @@
     <t xml:space="preserve">material</t>
   </si>
   <si>
-    <t xml:space="preserve">mottles</t>
-  </si>
-  <si>
-    <t xml:space="preserve">redox</t>
+    <t xml:space="preserve">mottle_abundance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mottle_size</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mottle_contrast</t>
   </si>
   <si>
     <t xml:space="preserve">notes</t>
@@ -151,9 +184,6 @@
     <t xml:space="preserve">3</t>
   </si>
   <si>
-    <t xml:space="preserve">2</t>
-  </si>
-  <si>
     <t xml:space="preserve">SiCL</t>
   </si>
   <si>
@@ -169,6 +199,12 @@
     <t xml:space="preserve">Few</t>
   </si>
   <si>
+    <t xml:space="preserve">Fine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Distinct</t>
+  </si>
+  <si>
     <t xml:space="preserve">Oxidized root channels; abrupt smooth lower boundary.</t>
   </si>
   <si>
@@ -196,6 +232,18 @@
     <t xml:space="preserve">hydric_ind_present: Yes / No — were any hydric soil indicators observed? | hydric_criterion_met: Yes / No / Marginal — overall hydric soil determination | soil_great_group: CSSC great group from field assessment (e.g. Humic Gleysol, Mesisol, Luvic Gleysol) — classify after field season if uncertain | additional_notes: free-text notes from the form footer</t>
   </si>
   <si>
+    <t xml:space="preserve">plots — physiography</t>
+  </si>
+  <si>
+    <t xml:space="preserve">slope_position: C=crest / U=upper / M=mid / L=lower / D=depression / Level | slope_pct: slope gradient in percent (0 = level; may exceed 100 on steep slopes) | aspect: downslope compass direction — N / NE / E / SE / S / SW / W / NW, or Flat where there is no aspect | drainage (CSSC 7-class): VR=very rapidly / R=rapidly / W=well / MW=moderately well / I=imperfectly / P=poorly / VP=very poorly drained | surface_stones: CSSC surface stoniness class S0 (nonstony) through S5 (exceedingly stony)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">horizons — horizon code</t>
+  </si>
+  <si>
+    <t xml:space="preserve">horizon: choose from the dropdown of standard CSSC horizon designations (organic L / F / H / LFH / O / Of / Om / Oh; A horizons Ah / Ahe / Ahg / Ae / Aeg / Ap / AB; B horizons Bm / Bg / Bgf / Bf / Bfg / Bh / Bhf / Bt / Btg / Btjg / Bnt / Bss; C horizons C / Cg / Ck / Ckg / Cca / Css; R; W). Letters only — the protocol does not use numbered subdivisions. The list is drawn from data-raw/cssc_great_groups.csv plus common wetland horizons; if a horizon you need is missing, add it to the dropdown in create_soils_template.R.</t>
+  </si>
+  <si>
     <t xml:space="preserve">horizons — Munsell colour</t>
   </si>
   <si>
@@ -220,10 +268,16 @@
     <t xml:space="preserve">Von Post humification scale H1–H10 for organic horizons. H1-H3 = Fibric (&gt;40% fibre, raw peat); H4-H6 = Mesic (17-40% fibre, moderately decomposed); H7-H10 = Humic (&lt;17% fibre, well decomposed). Leave blank for mineral horizons.</t>
   </si>
   <si>
+    <t xml:space="preserve">horizons — mottles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Record mottles / redoximorphic features in three separate columns, matching the field-form checkbox groups: mottle_abundance: None / Few / Common / Many (form codes None / Few / Com / Many) | mottle_size: Fine / Medium / Coarse (form codes F / M / C) | mottle_contrast: Faint / Distinct / Prominent (form codes F / D / P). Set mottle_abundance to None (or leave the row blank) when no mottles are present; leave mottle_size and mottle_contrast blank in that case.</t>
+  </si>
+  <si>
     <t xml:space="preserve">DO NOT COMPUTE</t>
   </si>
   <si>
-    <t xml:space="preserve">The following are derived by R in 03_transform.Rmd — do NOT enter manually: peat_depth_cm (sum of Peat/Muck horizon thicknesses), organic_fibre_class (from von_post: Fi/Me/Hu), hydric_indicators list (from colour, mottles, redox, horizon sequence), cssc_great_group_confirmed (CSSC classification from horizon sequence).</t>
+    <t xml:space="preserve">The following are derived by R in 03_transform.Rmd — do NOT enter manually: peat_depth_cm (sum of Peat/Muck horizon thicknesses), organic_fibre_class (from von_post: Fi/Me/Hu), hydric_indicators list (from colour, mottle characteristics, horizon sequence), cssc_great_group_confirmed (CSSC classification from horizon sequence).</t>
   </si>
 </sst>
 </file>
@@ -641,9 +695,14 @@
     <col min="8" max="8" width="13.71" hidden="0" customWidth="1"/>
     <col min="9" max="9" width="13.71" hidden="0" customWidth="1"/>
     <col min="10" max="10" width="13.71" hidden="0" customWidth="1"/>
-    <col min="11" max="11" width="13.71" hidden="0" customWidth="1"/>
-    <col min="12" max="12" width="24.71" hidden="0" customWidth="1"/>
-    <col min="13" max="13" width="44.71" hidden="0" customWidth="1"/>
+    <col min="11" max="11" width="9.71" hidden="0" customWidth="1"/>
+    <col min="12" max="12" width="9.71" hidden="0" customWidth="1"/>
+    <col min="13" max="13" width="9.71" hidden="0" customWidth="1"/>
+    <col min="14" max="14" width="13.71" hidden="0" customWidth="1"/>
+    <col min="15" max="15" width="13.71" hidden="0" customWidth="1"/>
+    <col min="16" max="16" width="13.71" hidden="0" customWidth="1"/>
+    <col min="17" max="17" width="24.71" hidden="0" customWidth="1"/>
+    <col min="18" max="18" width="44.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -662,6 +721,11 @@
       <c r="K1" s="1"/>
       <c r="L1" s="1"/>
       <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
+      <c r="Q1" s="1"/>
+      <c r="R1" s="1"/>
     </row>
     <row r="2" ht="38" customHeight="1">
       <c r="A2" s="2" t="s">
@@ -703,54 +767,87 @@
       <c r="M2" s="2" t="s">
         <v>13</v>
       </c>
+      <c r="N2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="R2" s="2" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>25</v>
+        <v>31</v>
+      </c>
+      <c r="N3" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="O3" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="P3" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q3" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="R3" s="3" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A1:R1"/>
   </mergeCells>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4:F1003">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4:K1003">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -758,7 +855,7 @@
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="7">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>"Pit,Probe"</xm:f>
@@ -769,13 +866,37 @@
           <x14:formula1>
             <xm:f>"Yes,No"</xm:f>
           </x14:formula1>
+          <xm:sqref>O4:O1003</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>"Yes,No,Marginal"</xm:f>
+          </x14:formula1>
+          <xm:sqref>P4:P1003</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>"C,U,M,L,D,Level"</xm:f>
+          </x14:formula1>
           <xm:sqref>J4:J1003</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
-            <xm:f>"Yes,No,Marginal"</xm:f>
-          </x14:formula1>
-          <xm:sqref>K4:K1003</xm:sqref>
+            <xm:f>"N,NE,E,SE,S,SW,W,NW,Flat"</xm:f>
+          </x14:formula1>
+          <xm:sqref>L4:L1003</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>"VR,R,W,MW,I,P,VP"</xm:f>
+          </x14:formula1>
+          <xm:sqref>M4:M1003</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>"S0,S1,S2,S3,S4,S5"</xm:f>
+          </x14:formula1>
+          <xm:sqref>N4:N1003</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -803,14 +924,15 @@
     <col min="10" max="10" width="9.71" hidden="0" customWidth="1"/>
     <col min="11" max="11" width="8.71" hidden="0" customWidth="1"/>
     <col min="12" max="12" width="9.71" hidden="0" customWidth="1"/>
-    <col min="13" max="13" width="9.71" hidden="0" customWidth="1"/>
-    <col min="14" max="14" width="9.71" hidden="0" customWidth="1"/>
-    <col min="15" max="15" width="44.71" hidden="0" customWidth="1"/>
+    <col min="13" max="13" width="11.71" hidden="0" customWidth="1"/>
+    <col min="14" max="14" width="10.71" hidden="0" customWidth="1"/>
+    <col min="15" max="15" width="11.71" hidden="0" customWidth="1"/>
+    <col min="16" max="16" width="44.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -826,6 +948,7 @@
       <c r="M1" s="1"/>
       <c r="N1" s="1"/>
       <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
     </row>
     <row r="2" ht="38" customHeight="1">
       <c r="A2" s="2" t="s">
@@ -835,95 +958,101 @@
         <v>3</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="O2" s="2" t="s">
-        <v>39</v>
+        <v>49</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>41</v>
+        <v>52</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>45</v>
+        <v>29</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>48</v>
+        <v>58</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="N3" s="3" t="s">
-        <v>50</v>
+        <v>61</v>
       </c>
       <c r="O3" s="3" t="s">
-        <v>51</v>
+        <v>62</v>
+      </c>
+      <c r="P3" s="3" t="s">
+        <v>63</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A1:P1"/>
   </mergeCells>
   <dataValidations count="4">
     <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4:D1003">
@@ -945,7 +1074,13 @@
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="6">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="8">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>"L,F,H,LFH,O,Of,Om,Oh,Ah,Ahe,Ahg,Ae,Aeg,Ap,AB,Bm,Bg,Bgf,Bf,Bfg,Bh,Bhf,Bt,Btg,Btjg,Bnt,Bss,C,Cg,Ck,Ckg,Cca,Css,R,W"</xm:f>
+          </x14:formula1>
+          <xm:sqref>C4:C1003</xm:sqref>
+        </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>"S,LS,SL,L,SiL,Si,SCL,CL,SiCL,SC,SiC,C,Muck,Peat"</xm:f>
@@ -972,15 +1107,21 @@
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
-            <xm:f>"None,Few,Com,Many"</xm:f>
+            <xm:f>"None,Few,Common,Many"</xm:f>
           </x14:formula1>
           <xm:sqref>M4:M1003</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
-            <xm:f>"None,Few,Com,Many"</xm:f>
+            <xm:f>"Fine,Medium,Coarse"</xm:f>
           </x14:formula1>
           <xm:sqref>N4:N1003</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>"Faint,Distinct,Prominent"</xm:f>
+          </x14:formula1>
+          <xm:sqref>O4:O1003</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -1002,74 +1143,98 @@
   <sheetData>
     <row r="1" ht="44" customHeight="1">
       <c r="A1" s="4" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>53</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="4" t="s">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>55</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" ht="60" customHeight="1">
       <c r="A3" s="4" t="s">
-        <v>56</v>
+        <v>68</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>57</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4" ht="72" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="5" ht="60" customHeight="1">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="5" ht="72" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="6" ht="72" customHeight="1">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="6" ht="96" customHeight="1">
       <c r="A6" s="4" t="s">
-        <v>62</v>
+        <v>74</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>63</v>
+        <v>75</v>
       </c>
     </row>
     <row r="7" ht="60" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>64</v>
+        <v>76</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>65</v>
+        <v>77</v>
       </c>
     </row>
     <row r="8" ht="72" customHeight="1">
       <c r="A8" s="4" t="s">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="9" ht="72" customHeight="1">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="9" ht="60" customHeight="1">
       <c r="A9" s="4" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>69</v>
+        <v>81</v>
+      </c>
+    </row>
+    <row r="10" ht="72" customHeight="1">
+      <c r="A10" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="11" ht="72" customHeight="1">
+      <c r="A11" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="12" ht="72" customHeight="1">
+      <c r="A12" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>